<commit_message>
data: update records 2026-10-20
</commit_message>
<xml_diff>
--- a/public/records.xlsx
+++ b/public/records.xlsx
@@ -4357,33 +4357,33 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Бабинич Егор</t>
+          <t>Вековищев Григорий</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>7:39.26</t>
+          <t>7:38.29</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>459.26</t>
+          <t>458.29</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Казань</t>
+          <t>Астана</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>2025-11-11</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -7383,23 +7383,23 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Бабинич Егор</t>
+          <t>Вековищев Григорий</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>7:39.26</t>
+          <t>7:38.29</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Казань</t>
+          <t>Астана</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>17.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>